<commit_message>
Reconcile handoff package: security gate, workflow archival, artifact fixes
- Archive stale AWS ECS deploy workflows (push triggers disabled; were
  failing red on every push — real deploys are Railway+Vercel)
- Security: classify pre-launch gate OPEN — ENVIRONMENT=staging keeps
  dev-token reachable; PAYMOB_SECRET_KEY is sk_test (sandbox rail)
- Correct Paymob Accept claims: sandbox-verified, live key pending
- Mobile terminology: READY TO START PHASE 1, not launch ready
- Document deterministic migration release sequence
- Regenerate legal EN/AR (funds-holding wording) + marketing (Arabic
  font fix, bank-transfer framing) + workbook v4

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/StayOS_Technical_Developer_Handoff_Workbook_2026-10-04_v4.xlsx
+++ b/StayOS_Technical_Developer_Handoff_Workbook_2026-10-04_v4.xlsx
@@ -437,11 +437,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="57" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -487,7 +487,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-04 (v4 — supersedes v3)</t>
+          <t>2026-10-04 (v4 — reconciled)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -499,12 +499,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Final handoff commit</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CLOSED — founder acceptance, web-amber-pi-98.vercel.app</t>
+          <t>main HEAD at package time — see manifest/git log</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -516,12 +516,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1644 passed, ~80.5% coverage</t>
+          <t>CLOSED — founder acceptance, web-amber-pi-98.vercel.app</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -533,12 +533,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Web tests</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>222 passed; tsc+build clean</t>
+          <t>1644 passed, 80.46% coverage</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -550,12 +550,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Web tests</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>READY — Phase 4 start approved</t>
+          <t>222 passed; tsc clean</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -567,15 +567,32 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>READY TO START PHASE 1 — NOT LAUNCH READY</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Railway (api/worker/beat) + Vercel (web)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Railway (api/worker/beat) + Vercel (web); ENVIRONMENT=staging — pre-launch gate open</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>CURRENT</t>
         </is>
@@ -596,7 +613,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="51" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -619,7 +636,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LIVE</t>
+          <t>SANDBOX — sk_test key; flow verified, no real money; live key = external blocker</t>
         </is>
       </c>
     </row>
@@ -691,7 +708,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>placeholder details unset</t>
+          <t>implemented; placeholder details unset</t>
         </is>
       </c>
     </row>
@@ -706,11 +723,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -733,7 +750,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1644 pass</t>
+          <t>1644 pass, 80.46% cov</t>
         </is>
       </c>
     </row>
@@ -782,6 +799,18 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>db ok, redis ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>auth boundary</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>unauthed 401; staff-only 403</t>
         </is>
       </c>
     </row>
@@ -796,11 +825,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -824,12 +853,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Screens</t>
+          <t>Verdict</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>28 (guest+host)</t>
+          <t>READY TO START PHASE 1 — NOT LAUNCH READY</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -841,12 +870,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Endpoints</t>
+          <t>Screens</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>25/25 resolve</t>
+          <t>28 (guest+host)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -858,68 +887,85 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Endpoints</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>WhatsApp-only screen</t>
+          <t>25/25 resolve</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>P1 in-app threads</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Host filters</t>
+          <t>Support</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>/host/reservations basic</t>
+          <t>WhatsApp-only screen</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>P1 adopt /host/bookings params</t>
+          <t>P1 in-app threads</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Help</t>
+          <t>Host filters</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>/host/reservations basic</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1 adopt /host/bookings params</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Help</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Builds</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>preview APK + CI</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>P1 prod EAS profile</t>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>P1 prod EAS profile; P2 iOS</t>
         </is>
       </c>
     </row>
@@ -934,10 +980,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -956,19 +1002,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Paymob Payouts unprovisioned</t>
+          <t>ENVIRONMENT=staging + dev-token + sk_test</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>EXTERNAL BLOCKER</t>
+          <t>PRE-LAUNCH GATE — OPEN</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sumsub not activated</t>
+          <t>Paymob Payouts unprovisioned</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -980,46 +1026,58 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e-invoice/e-receipt</t>
+          <t>Sumsub not activated</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LEGAL/ACCOUNTING OPEN ITEM</t>
+          <t>EXTERNAL BLOCKER</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Stale AWS workflows</t>
+          <t>Live Paymob Accept key</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CURRENT — flag for removal</t>
+          <t>EXTERNAL BLOCKER</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Manual transfer placeholders</t>
+          <t>e-invoice/e-receipt</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CURRENT — needs real details</t>
+          <t>LEGAL/ACCOUNTING OPEN ITEM</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Manual transfer placeholders</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CURRENT — needs real details</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Mobile support/help UI</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>CURRENT — Phase 1 scope</t>
         </is>
@@ -1036,11 +1094,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="49" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1063,7 +1121,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>STAYOS_SOURCE_HANDOFF_2026-10-04.zip</t>
+          <t>STAYOS_SOURCE_HANDOFF_2026-10-04.zip (+ .sha256 sidecar)</t>
         </is>
       </c>
     </row>
@@ -1075,53 +1133,65 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>STAYOS_GIT_HANDOFF_2026-10-04.bundle</t>
+          <t>STAYOS_GIT_HANDOFF_2026-10-04.bundle (+ .sha256 sidecar)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Handbook</t>
+          <t>Rendered manifest</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>docs/handoff/ (59 files)</t>
+          <t>inside ZIP + repo root</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Workbook</t>
+          <t>Handbook</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>this file (v4)</t>
+          <t>docs/handoff/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Legal pack</t>
+          <t>Workbook</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>StayOS_Legal_*_2026-10-04_v4{,_AR}.pdf</t>
+          <t>this file (v4)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Legal pack</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>StayOS_Legal_*_2026-10-04_v4{,_AR}.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>StayOS_Marketing_Launch_Brief_V3_PRODUCT_UI.pdf</t>
         </is>
@@ -1138,11 +1208,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1160,12 +1230,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Pre-launch</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Close security gate: live Paymob key → ENVIRONMENT=production (33_SECURITY.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>PHASE 4 — MOBILE</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Execute docs/handoff/MOBILE_PHASE_1_EXECUTION_PLAN.md — support inbox, host filter parity, EAS prod profile</t>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Execute docs/handoff/MOBILE_PHASE_1_EXECUTION_PLAN.md</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1267,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="29" customWidth="1" min="2" max="2"/>
-    <col width="47" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1269,7 +1351,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>through 053_support_conversations</t>
+          <t>through 053_support_conversations; NOT auto-applied on deploy</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1663,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1857,7 +1939,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1895,11 +1977,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1946,19 +2028,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>alembic via railway connect tunnel</t>
+          <t>EXPLICIT step — railway connect tunnel + alembic upgrade head; NOT automatic</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Stale CI</t>
+          <t>Release order</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>deploy-prod/staging.yml → AWS ECS; FAIL on push — not the deploy path</t>
+          <t>code deploy → migration → verify → worker/beat → web acceptance</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AWS workflows</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>deploy-prod/staging.yml ARCHIVED 2026-10-04 — push triggers disabled</t>
         </is>
       </c>
     </row>
@@ -1973,11 +2067,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1995,36 +2089,60 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AuthZ</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>server-side role+permission+ownership</t>
+          <t>PRE-LAUNCH GATE OPEN — not GREEN</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Gate findings</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tracked tree + history scan clean; placeholders only</t>
+          <t>ENVIRONMENT=staging on prod; dev-token reachable (mints JWT for known user_id); PAYMOB_SECRET_KEY is sk_test (sandbox)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Flag</t>
+          <t>Remediation</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>prod service ENVIRONMENT=staging → dev-token reachable; tighten pre-launch</t>
+          <t>live Paymob key → real PAYMENT_BANK_* → ENVIRONMENT=production (fail-closed order) → verify dev-token 404</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AuthZ</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>server-side role+permission+ownership — verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Secrets</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tracked tree + history scan clean; placeholders only</t>
         </is>
       </c>
     </row>

</xml_diff>